<commit_message>
Integración exitosa de Webpay, inventario en Excel y sección de pedidos
</commit_message>
<xml_diff>
--- a/INVENTARIOREAL2026.xlsx
+++ b/INVENTARIOREAL2026.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ext_jmena\OneDrive - Falabella\Escritorio\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ext_jmena\OneDrive - Falabella\Escritorio\distribuidora2\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1113" uniqueCount="568">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1114" uniqueCount="569">
   <si>
     <t>CODIGO</t>
   </si>
@@ -1723,6 +1723,9 @@
   </si>
   <si>
     <t>HUEVO 1ERA 6 BANDEJAS (180 UN) SOLO DESPACHO</t>
+  </si>
+  <si>
+    <t>stock</t>
   </si>
 </sst>
 </file>
@@ -1767,7 +1770,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -1790,12 +1793,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1804,6 +1818,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="42" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2109,7 +2129,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E278"/>
+  <dimension ref="A1:F278"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
@@ -2119,7 +2139,7 @@
     <col min="5" max="5" width="8.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2135,8 +2155,11 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F1" s="4" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -2152,8 +2175,11 @@
       <c r="E2" s="3">
         <v>5520</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F2" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>9</v>
       </c>
@@ -2169,8 +2195,11 @@
       <c r="E3" s="3">
         <v>5520</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F3" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
@@ -2186,8 +2215,11 @@
       <c r="E4" s="3">
         <v>5520</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F4" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>13</v>
       </c>
@@ -2203,8 +2235,11 @@
       <c r="E5" s="3">
         <v>5520</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F5" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
@@ -2220,8 +2255,11 @@
       <c r="E6" s="3">
         <v>6540</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F6" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>17</v>
       </c>
@@ -2237,8 +2275,11 @@
       <c r="E7" s="3">
         <v>6540</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F7" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>19</v>
       </c>
@@ -2254,8 +2295,11 @@
       <c r="E8" s="3">
         <v>4000</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F8" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>21</v>
       </c>
@@ -2271,8 +2315,11 @@
       <c r="E9" s="3">
         <v>4000</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F9" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>23</v>
       </c>
@@ -2288,8 +2335,11 @@
       <c r="E10" s="3">
         <v>4000</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F10" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>25</v>
       </c>
@@ -2305,8 +2355,11 @@
       <c r="E11" s="3">
         <v>4000</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F11" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>27</v>
       </c>
@@ -2322,8 +2375,11 @@
       <c r="E12" s="3">
         <v>10200</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F12" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>30</v>
       </c>
@@ -2339,8 +2395,11 @@
       <c r="E13" s="3">
         <v>10200</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F13" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>32</v>
       </c>
@@ -2356,8 +2415,11 @@
       <c r="E14" s="3">
         <v>10200</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F14" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>34</v>
       </c>
@@ -2373,8 +2435,11 @@
       <c r="E15" s="3">
         <v>10200</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F15" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>36</v>
       </c>
@@ -2390,8 +2455,11 @@
       <c r="E16" s="3">
         <v>10200</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F16" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>38</v>
       </c>
@@ -2407,8 +2475,11 @@
       <c r="E17" s="3">
         <v>10200</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F17" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>40</v>
       </c>
@@ -2424,8 +2495,11 @@
       <c r="E18" s="3">
         <v>10200</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F18" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>42</v>
       </c>
@@ -2441,8 +2515,11 @@
       <c r="E19" s="3">
         <v>10200</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F19" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>44</v>
       </c>
@@ -2458,8 +2535,11 @@
       <c r="E20" s="3">
         <v>11200</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F20" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>46</v>
       </c>
@@ -2475,8 +2555,11 @@
       <c r="E21" s="3">
         <v>11200</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F21" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>48</v>
       </c>
@@ -2492,8 +2575,11 @@
       <c r="E22" s="3">
         <v>11200</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F22" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>50</v>
       </c>
@@ -2509,8 +2595,11 @@
       <c r="E23" s="3">
         <v>11200</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F23" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>52</v>
       </c>
@@ -2526,8 +2615,11 @@
       <c r="E24" s="3">
         <v>11200</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F24" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>54</v>
       </c>
@@ -2543,8 +2635,11 @@
       <c r="E25" s="3">
         <v>11200</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F25" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>56</v>
       </c>
@@ -2560,8 +2655,11 @@
       <c r="E26" s="3">
         <v>7260</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F26" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>58</v>
       </c>
@@ -2577,8 +2675,11 @@
       <c r="E27" s="3">
         <v>7260</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F27" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>60</v>
       </c>
@@ -2594,8 +2695,11 @@
       <c r="E28" s="3">
         <v>7260</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F28" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>62</v>
       </c>
@@ -2611,8 +2715,11 @@
       <c r="E29" s="3">
         <v>5280</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F29" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>64</v>
       </c>
@@ -2628,8 +2735,11 @@
       <c r="E30" s="3">
         <v>5280</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F30" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>66</v>
       </c>
@@ -2645,8 +2755,11 @@
       <c r="E31" s="3">
         <v>5280</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F31" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>68</v>
       </c>
@@ -2662,8 +2775,11 @@
       <c r="E32" s="3">
         <v>12990</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F32" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>70</v>
       </c>
@@ -2679,8 +2795,11 @@
       <c r="E33" s="3">
         <v>12990</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F33" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>72</v>
       </c>
@@ -2696,8 +2815,11 @@
       <c r="E34" s="3">
         <v>12990</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F34" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>74</v>
       </c>
@@ -2713,8 +2835,11 @@
       <c r="E35" s="3">
         <v>12990</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F35" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>76</v>
       </c>
@@ -2730,8 +2855,11 @@
       <c r="E36" s="3">
         <v>12990</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F36" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>78</v>
       </c>
@@ -2747,8 +2875,11 @@
       <c r="E37" s="3">
         <v>12990</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F37" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>80</v>
       </c>
@@ -2764,8 +2895,11 @@
       <c r="E38" s="3">
         <v>13545</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F38" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>82</v>
       </c>
@@ -2781,8 +2915,11 @@
       <c r="E39" s="3">
         <v>13545</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F39" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
         <v>84</v>
       </c>
@@ -2798,8 +2935,11 @@
       <c r="E40" s="3">
         <v>13545</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F40" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>86</v>
       </c>
@@ -2815,8 +2955,11 @@
       <c r="E41" s="3">
         <v>13545</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F41" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>88</v>
       </c>
@@ -2832,8 +2975,11 @@
       <c r="E42" s="3">
         <v>13545</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F42" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
         <v>90</v>
       </c>
@@ -2849,8 +2995,11 @@
       <c r="E43" s="3">
         <v>13545</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F43" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
         <v>92</v>
       </c>
@@ -2866,8 +3015,11 @@
       <c r="E44" s="3">
         <v>9498</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F44" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
         <v>94</v>
       </c>
@@ -2883,8 +3035,11 @@
       <c r="E45" s="3">
         <v>9498</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F45" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
         <v>96</v>
       </c>
@@ -2900,8 +3055,11 @@
       <c r="E46" s="3">
         <v>9498</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F46" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
         <v>98</v>
       </c>
@@ -2917,8 +3075,11 @@
       <c r="E47" s="3">
         <v>9498</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F47" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
         <v>100</v>
       </c>
@@ -2934,8 +3095,11 @@
       <c r="E48" s="3">
         <v>9498</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F48" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
         <v>102</v>
       </c>
@@ -2951,8 +3115,11 @@
       <c r="E49" s="3">
         <v>9498</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F49" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
         <v>104</v>
       </c>
@@ -2968,8 +3135,11 @@
       <c r="E50" s="3">
         <v>9498</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F50" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
         <v>106</v>
       </c>
@@ -2985,8 +3155,11 @@
       <c r="E51" s="3">
         <v>9498</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F51" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
         <v>108</v>
       </c>
@@ -3002,8 +3175,11 @@
       <c r="E52" s="3">
         <v>12080</v>
       </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F52" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" s="2" t="s">
         <v>110</v>
       </c>
@@ -3019,8 +3195,11 @@
       <c r="E53" s="3">
         <v>12080</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F53" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
         <v>112</v>
       </c>
@@ -3036,8 +3215,11 @@
       <c r="E54" s="3">
         <v>12080</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F54" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
         <v>114</v>
       </c>
@@ -3053,8 +3235,11 @@
       <c r="E55" s="3">
         <v>12080</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F55" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
         <v>116</v>
       </c>
@@ -3070,8 +3255,11 @@
       <c r="E56" s="3">
         <v>12080</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F56" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
         <v>118</v>
       </c>
@@ -3087,8 +3275,11 @@
       <c r="E57" s="3">
         <v>12080</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F57" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
         <v>120</v>
       </c>
@@ -3104,8 +3295,11 @@
       <c r="E58" s="3">
         <v>12080</v>
       </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F58" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
         <v>122</v>
       </c>
@@ -3121,8 +3315,11 @@
       <c r="E59" s="3">
         <v>12080</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F59" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>124</v>
       </c>
@@ -3138,8 +3335,11 @@
       <c r="E60" s="3">
         <v>12080</v>
       </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F60" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
         <v>126</v>
       </c>
@@ -3155,8 +3355,11 @@
       <c r="E61" s="3">
         <v>3780</v>
       </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F61" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
         <v>128</v>
       </c>
@@ -3172,8 +3375,11 @@
       <c r="E62" s="3">
         <v>3780</v>
       </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F62" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" s="2" t="s">
         <v>130</v>
       </c>
@@ -3189,8 +3395,11 @@
       <c r="E63" s="3">
         <v>3780</v>
       </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F63" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" s="2" t="s">
         <v>132</v>
       </c>
@@ -3206,8 +3415,11 @@
       <c r="E64" s="3">
         <v>3780</v>
       </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F64" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" s="2" t="s">
         <v>134</v>
       </c>
@@ -3223,8 +3435,11 @@
       <c r="E65" s="3">
         <v>3780</v>
       </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F65" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" s="2" t="s">
         <v>136</v>
       </c>
@@ -3240,8 +3455,11 @@
       <c r="E66" s="3">
         <v>3780</v>
       </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F66" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" s="2" t="s">
         <v>138</v>
       </c>
@@ -3257,8 +3475,11 @@
       <c r="E67" s="3">
         <v>3780</v>
       </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F67" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68" s="2" t="s">
         <v>140</v>
       </c>
@@ -3274,8 +3495,11 @@
       <c r="E68" s="3">
         <v>3780</v>
       </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F68" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69" s="2" t="s">
         <v>142</v>
       </c>
@@ -3291,8 +3515,11 @@
       <c r="E69" s="3">
         <v>3780</v>
       </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F69" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70" s="2" t="s">
         <v>144</v>
       </c>
@@ -3308,8 +3535,11 @@
       <c r="E70" s="3">
         <v>3780</v>
       </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F70" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71" s="2" t="s">
         <v>146</v>
       </c>
@@ -3325,8 +3555,11 @@
       <c r="E71" s="3">
         <v>11526</v>
       </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F71" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" s="2" t="s">
         <v>148</v>
       </c>
@@ -3342,8 +3575,11 @@
       <c r="E72" s="3">
         <v>11526</v>
       </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F72" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73" s="2" t="s">
         <v>150</v>
       </c>
@@ -3359,8 +3595,11 @@
       <c r="E73" s="3">
         <v>11526</v>
       </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F73" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" s="2" t="s">
         <v>152</v>
       </c>
@@ -3376,8 +3615,11 @@
       <c r="E74" s="3">
         <v>11526</v>
       </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F74" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75" s="2" t="s">
         <v>154</v>
       </c>
@@ -3393,8 +3635,11 @@
       <c r="E75" s="3">
         <v>11526</v>
       </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F75" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76" s="2" t="s">
         <v>156</v>
       </c>
@@ -3410,8 +3655,11 @@
       <c r="E76" s="3">
         <v>10516</v>
       </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F76" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77" s="2" t="s">
         <v>158</v>
       </c>
@@ -3427,8 +3675,11 @@
       <c r="E77" s="3">
         <v>10516</v>
       </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F77" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A78" s="2" t="s">
         <v>160</v>
       </c>
@@ -3444,8 +3695,11 @@
       <c r="E78" s="3">
         <v>10516</v>
       </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F78" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A79" s="2" t="s">
         <v>162</v>
       </c>
@@ -3461,8 +3715,11 @@
       <c r="E79" s="3">
         <v>10516</v>
       </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F79" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A80" s="2" t="s">
         <v>164</v>
       </c>
@@ -3478,8 +3735,11 @@
       <c r="E80" s="3">
         <v>10516</v>
       </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F80" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A81" s="2" t="s">
         <v>166</v>
       </c>
@@ -3495,8 +3755,11 @@
       <c r="E81" s="3">
         <v>10516</v>
       </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F81" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A82" s="2" t="s">
         <v>168</v>
       </c>
@@ -3512,8 +3775,11 @@
       <c r="E82" s="3">
         <v>10516</v>
       </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F82" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A83" s="2" t="s">
         <v>170</v>
       </c>
@@ -3529,8 +3795,11 @@
       <c r="E83" s="3">
         <v>10516</v>
       </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F83" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A84" s="2" t="s">
         <v>172</v>
       </c>
@@ -3546,8 +3815,11 @@
       <c r="E84" s="3">
         <v>7521</v>
       </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F84" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A85" s="2" t="s">
         <v>174</v>
       </c>
@@ -3563,8 +3835,11 @@
       <c r="E85" s="3">
         <v>7521</v>
       </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F85" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A86" s="2" t="s">
         <v>176</v>
       </c>
@@ -3580,8 +3855,11 @@
       <c r="E86" s="3">
         <v>7521</v>
       </c>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F86" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A87" s="2" t="s">
         <v>178</v>
       </c>
@@ -3597,8 +3875,11 @@
       <c r="E87" s="3">
         <v>7521</v>
       </c>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F87" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A88" s="2" t="s">
         <v>180</v>
       </c>
@@ -3614,8 +3895,11 @@
       <c r="E88" s="3">
         <v>7521</v>
       </c>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F88" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A89" s="2" t="s">
         <v>182</v>
       </c>
@@ -3631,8 +3915,11 @@
       <c r="E89" s="3">
         <v>7521</v>
       </c>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F89" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A90" s="2" t="s">
         <v>184</v>
       </c>
@@ -3648,8 +3935,11 @@
       <c r="E90" s="3">
         <v>7521</v>
       </c>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F90" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A91" s="2" t="s">
         <v>186</v>
       </c>
@@ -3665,8 +3955,11 @@
       <c r="E91" s="3">
         <v>7521</v>
       </c>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F91" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A92" s="2" t="s">
         <v>188</v>
       </c>
@@ -3682,8 +3975,11 @@
       <c r="E92" s="3">
         <v>15200</v>
       </c>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F92" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A93" s="2" t="s">
         <v>190</v>
       </c>
@@ -3699,8 +3995,11 @@
       <c r="E93" s="3">
         <v>20760</v>
       </c>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F93" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A94" s="2" t="s">
         <v>192</v>
       </c>
@@ -3716,8 +4015,11 @@
       <c r="E94" s="3">
         <v>25920</v>
       </c>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F94" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A95" s="2" t="s">
         <v>194</v>
       </c>
@@ -3733,8 +4035,11 @@
       <c r="E95" s="3">
         <v>11160</v>
       </c>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F95" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A96" s="2" t="s">
         <v>196</v>
       </c>
@@ -3750,8 +4055,11 @@
       <c r="E96" s="3">
         <v>11160</v>
       </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F96" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A97" s="2" t="s">
         <v>198</v>
       </c>
@@ -3767,8 +4075,11 @@
       <c r="E97" s="3">
         <v>11160</v>
       </c>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F97" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A98" s="2" t="s">
         <v>200</v>
       </c>
@@ -3784,8 +4095,11 @@
       <c r="E98" s="3">
         <v>9120</v>
       </c>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F98" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A99" s="2" t="s">
         <v>202</v>
       </c>
@@ -3801,8 +4115,11 @@
       <c r="E99" s="3">
         <v>9120</v>
       </c>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F99" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A100" s="2" t="s">
         <v>204</v>
       </c>
@@ -3818,8 +4135,11 @@
       <c r="E100" s="3">
         <v>9120</v>
       </c>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F100" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A101" s="2" t="s">
         <v>206</v>
       </c>
@@ -3835,8 +4155,11 @@
       <c r="E101" s="3">
         <v>9120</v>
       </c>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F101" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A102" s="2" t="s">
         <v>208</v>
       </c>
@@ -3852,8 +4175,11 @@
       <c r="E102" s="3">
         <v>9120</v>
       </c>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F102" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A103" s="2" t="s">
         <v>210</v>
       </c>
@@ -3869,8 +4195,11 @@
       <c r="E103" s="3">
         <v>9120</v>
       </c>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F103" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A104" s="2" t="s">
         <v>212</v>
       </c>
@@ -3886,8 +4215,11 @@
       <c r="E104" s="3">
         <v>9120</v>
       </c>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F104" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A105" s="2" t="s">
         <v>214</v>
       </c>
@@ -3903,8 +4235,11 @@
       <c r="E105" s="3">
         <v>9120</v>
       </c>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F105" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A106" s="2" t="s">
         <v>216</v>
       </c>
@@ -3920,8 +4255,11 @@
       <c r="E106" s="3">
         <v>9120</v>
       </c>
-    </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F106" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A107" s="2" t="s">
         <v>218</v>
       </c>
@@ -3937,8 +4275,11 @@
       <c r="E107" s="3">
         <v>9120</v>
       </c>
-    </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F107" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A108" s="2" t="s">
         <v>220</v>
       </c>
@@ -3954,8 +4295,11 @@
       <c r="E108" s="3">
         <v>9120</v>
       </c>
-    </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F108" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A109" s="2" t="s">
         <v>222</v>
       </c>
@@ -3971,8 +4315,11 @@
       <c r="E109" s="3">
         <v>9120</v>
       </c>
-    </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F109" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A110" s="2" t="s">
         <v>224</v>
       </c>
@@ -3988,8 +4335,11 @@
       <c r="E110" s="3">
         <v>9120</v>
       </c>
-    </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F110" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A111" s="2" t="s">
         <v>226</v>
       </c>
@@ -4005,8 +4355,11 @@
       <c r="E111" s="3">
         <v>9120</v>
       </c>
-    </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F111" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A112" s="2" t="s">
         <v>228</v>
       </c>
@@ -4022,8 +4375,11 @@
       <c r="E112" s="3">
         <v>9120</v>
       </c>
-    </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F112" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A113" s="2" t="s">
         <v>230</v>
       </c>
@@ -4039,8 +4395,11 @@
       <c r="E113" s="3">
         <v>9120</v>
       </c>
-    </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F113" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A114" s="2" t="s">
         <v>232</v>
       </c>
@@ -4056,8 +4415,11 @@
       <c r="E114" s="3">
         <v>19920</v>
       </c>
-    </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F114" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A115" s="2" t="s">
         <v>234</v>
       </c>
@@ -4073,8 +4435,11 @@
       <c r="E115" s="3">
         <v>19920</v>
       </c>
-    </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F115" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A116" s="2" t="s">
         <v>236</v>
       </c>
@@ -4090,8 +4455,11 @@
       <c r="E116" s="3">
         <v>19920</v>
       </c>
-    </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F116" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A117" s="2" t="s">
         <v>238</v>
       </c>
@@ -4107,8 +4475,11 @@
       <c r="E117" s="3">
         <v>19920</v>
       </c>
-    </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F117" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A118" s="2" t="s">
         <v>240</v>
       </c>
@@ -4124,8 +4495,11 @@
       <c r="E118" s="3">
         <v>10250</v>
       </c>
-    </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F118" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A119" s="2" t="s">
         <v>243</v>
       </c>
@@ -4141,8 +4515,11 @@
       <c r="E119" s="3">
         <v>10250</v>
       </c>
-    </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F119" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A120" s="2" t="s">
         <v>245</v>
       </c>
@@ -4158,8 +4535,11 @@
       <c r="E120" s="3">
         <v>10250</v>
       </c>
-    </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F120" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A121" s="2" t="s">
         <v>247</v>
       </c>
@@ -4175,8 +4555,11 @@
       <c r="E121" s="3">
         <v>10250</v>
       </c>
-    </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F121" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A122" s="2" t="s">
         <v>249</v>
       </c>
@@ -4192,8 +4575,11 @@
       <c r="E122" s="3">
         <v>10250</v>
       </c>
-    </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F122" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A123" s="2" t="s">
         <v>251</v>
       </c>
@@ -4209,8 +4595,11 @@
       <c r="E123" s="3">
         <v>9888</v>
       </c>
-    </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F123" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A124" s="2" t="s">
         <v>253</v>
       </c>
@@ -4226,8 +4615,11 @@
       <c r="E124" s="3">
         <v>9888</v>
       </c>
-    </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F124" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A125" s="2" t="s">
         <v>255</v>
       </c>
@@ -4243,8 +4635,11 @@
       <c r="E125" s="3">
         <v>9888</v>
       </c>
-    </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F125" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A126" s="2" t="s">
         <v>257</v>
       </c>
@@ -4260,8 +4655,11 @@
       <c r="E126" s="3">
         <v>9888</v>
       </c>
-    </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F126" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A127" s="2" t="s">
         <v>259</v>
       </c>
@@ -4277,8 +4675,11 @@
       <c r="E127" s="3">
         <v>9888</v>
       </c>
-    </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F127" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A128" s="2" t="s">
         <v>261</v>
       </c>
@@ -4294,8 +4695,11 @@
       <c r="E128" s="3">
         <v>11880</v>
       </c>
-    </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F128" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A129" s="2" t="s">
         <v>263</v>
       </c>
@@ -4311,8 +4715,11 @@
       <c r="E129" s="3">
         <v>11880</v>
       </c>
-    </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F129" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A130" s="2" t="s">
         <v>265</v>
       </c>
@@ -4328,8 +4735,11 @@
       <c r="E130" s="3">
         <v>11880</v>
       </c>
-    </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F130" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A131" s="2" t="s">
         <v>267</v>
       </c>
@@ -4345,8 +4755,11 @@
       <c r="E131" s="3">
         <v>11880</v>
       </c>
-    </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F131" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A132" s="2" t="s">
         <v>269</v>
       </c>
@@ -4362,8 +4775,11 @@
       <c r="E132" s="3">
         <v>11880</v>
       </c>
-    </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F132" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A133" s="2" t="s">
         <v>271</v>
       </c>
@@ -4379,8 +4795,11 @@
       <c r="E133" s="3">
         <v>11880</v>
       </c>
-    </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F133" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A134" s="2" t="s">
         <v>273</v>
       </c>
@@ -4396,8 +4815,11 @@
       <c r="E134" s="3">
         <v>12642</v>
       </c>
-    </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F134" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A135" s="2" t="s">
         <v>275</v>
       </c>
@@ -4413,8 +4835,11 @@
       <c r="E135" s="3">
         <v>12642</v>
       </c>
-    </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F135" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A136" s="2" t="s">
         <v>277</v>
       </c>
@@ -4430,8 +4855,11 @@
       <c r="E136" s="3">
         <v>12642</v>
       </c>
-    </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F136" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A137" s="2" t="s">
         <v>279</v>
       </c>
@@ -4447,8 +4875,11 @@
       <c r="E137" s="3">
         <v>12642</v>
       </c>
-    </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F137" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A138" s="2" t="s">
         <v>281</v>
       </c>
@@ -4464,8 +4895,11 @@
       <c r="E138" s="3">
         <v>14850</v>
       </c>
-    </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F138" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A139" s="2" t="s">
         <v>283</v>
       </c>
@@ -4481,8 +4915,11 @@
       <c r="E139" s="3">
         <v>14850</v>
       </c>
-    </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F139" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A140" s="2" t="s">
         <v>285</v>
       </c>
@@ -4498,8 +4935,11 @@
       <c r="E140" s="3">
         <v>14850</v>
       </c>
-    </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F140" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="141" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A141" s="2" t="s">
         <v>287</v>
       </c>
@@ -4515,8 +4955,11 @@
       <c r="E141" s="3">
         <v>14850</v>
       </c>
-    </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F141" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="142" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A142" s="2" t="s">
         <v>289</v>
       </c>
@@ -4532,8 +4975,11 @@
       <c r="E142" s="3">
         <v>14850</v>
       </c>
-    </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F142" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="143" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A143" s="2" t="s">
         <v>291</v>
       </c>
@@ -4549,8 +4995,11 @@
       <c r="E143" s="3">
         <v>5040</v>
       </c>
-    </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F143" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="144" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A144" s="2" t="s">
         <v>293</v>
       </c>
@@ -4566,8 +5015,11 @@
       <c r="E144" s="3">
         <v>5040</v>
       </c>
-    </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F144" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="145" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A145" s="2" t="s">
         <v>295</v>
       </c>
@@ -4583,8 +5035,11 @@
       <c r="E145" s="3">
         <v>5040</v>
       </c>
-    </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F145" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="146" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A146" s="2" t="s">
         <v>297</v>
       </c>
@@ -4600,8 +5055,11 @@
       <c r="E146" s="3">
         <v>5040</v>
       </c>
-    </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F146" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="147" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A147" s="2" t="s">
         <v>299</v>
       </c>
@@ -4617,8 +5075,11 @@
       <c r="E147" s="3">
         <v>5760</v>
       </c>
-    </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F147" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="148" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A148" s="2" t="s">
         <v>301</v>
       </c>
@@ -4634,8 +5095,11 @@
       <c r="E148" s="3">
         <v>5760</v>
       </c>
-    </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F148" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="149" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A149" s="2" t="s">
         <v>303</v>
       </c>
@@ -4651,8 +5115,11 @@
       <c r="E149" s="3">
         <v>5760</v>
       </c>
-    </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F149" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="150" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A150" s="2" t="s">
         <v>305</v>
       </c>
@@ -4668,8 +5135,11 @@
       <c r="E150" s="3">
         <v>5760</v>
       </c>
-    </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F150" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A151" s="2" t="s">
         <v>307</v>
       </c>
@@ -4685,8 +5155,11 @@
       <c r="E151" s="3">
         <v>6540</v>
       </c>
-    </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F151" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="152" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A152" s="2" t="s">
         <v>309</v>
       </c>
@@ -4702,8 +5175,11 @@
       <c r="E152" s="3">
         <v>6540</v>
       </c>
-    </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F152" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="153" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A153" s="2" t="s">
         <v>311</v>
       </c>
@@ -4719,8 +5195,11 @@
       <c r="E153" s="3">
         <v>6540</v>
       </c>
-    </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F153" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="154" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A154" s="2" t="s">
         <v>313</v>
       </c>
@@ -4736,8 +5215,11 @@
       <c r="E154" s="3">
         <v>6540</v>
       </c>
-    </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F154" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="155" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A155" s="2" t="s">
         <v>315</v>
       </c>
@@ -4753,8 +5235,11 @@
       <c r="E155" s="3">
         <v>6540</v>
       </c>
-    </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F155" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="156" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A156" s="2" t="s">
         <v>317</v>
       </c>
@@ -4770,8 +5255,11 @@
       <c r="E156" s="3">
         <v>4680</v>
       </c>
-    </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F156" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="157" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A157" s="2" t="s">
         <v>319</v>
       </c>
@@ -4787,8 +5275,11 @@
       <c r="E157" s="3">
         <v>4680</v>
       </c>
-    </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F157" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="158" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A158" s="2" t="s">
         <v>321</v>
       </c>
@@ -4804,8 +5295,11 @@
       <c r="E158" s="3">
         <v>6900</v>
       </c>
-    </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F158" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="159" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A159" s="2" t="s">
         <v>323</v>
       </c>
@@ -4821,8 +5315,11 @@
       <c r="E159" s="3">
         <v>6900</v>
       </c>
-    </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F159" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="160" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A160" s="2" t="s">
         <v>325</v>
       </c>
@@ -4838,8 +5335,11 @@
       <c r="E160" s="3">
         <v>6480</v>
       </c>
-    </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F160" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="161" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A161" s="2" t="s">
         <v>327</v>
       </c>
@@ -4855,8 +5355,11 @@
       <c r="E161" s="3">
         <v>6480</v>
       </c>
-    </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F161" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="162" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A162" s="2" t="s">
         <v>329</v>
       </c>
@@ -4872,8 +5375,11 @@
       <c r="E162" s="3">
         <v>6480</v>
       </c>
-    </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F162" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="163" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A163" s="2" t="s">
         <v>331</v>
       </c>
@@ -4889,8 +5395,11 @@
       <c r="E163" s="3">
         <v>6480</v>
       </c>
-    </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F163" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="164" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A164" s="2" t="s">
         <v>333</v>
       </c>
@@ -4906,8 +5415,11 @@
       <c r="E164" s="3">
         <v>6480</v>
       </c>
-    </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F164" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="165" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A165" s="2" t="s">
         <v>335</v>
       </c>
@@ -4923,8 +5435,11 @@
       <c r="E165" s="3">
         <v>3900</v>
       </c>
-    </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F165" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="166" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A166" s="2" t="s">
         <v>337</v>
       </c>
@@ -4940,8 +5455,11 @@
       <c r="E166" s="3">
         <v>3900</v>
       </c>
-    </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F166" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="167" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A167" s="2" t="s">
         <v>339</v>
       </c>
@@ -4957,8 +5475,11 @@
       <c r="E167" s="3">
         <v>4428</v>
       </c>
-    </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F167" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="168" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A168" s="2" t="s">
         <v>341</v>
       </c>
@@ -4974,8 +5495,11 @@
       <c r="E168" s="3">
         <v>4428</v>
       </c>
-    </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F168" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="169" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A169" s="2" t="s">
         <v>343</v>
       </c>
@@ -4991,8 +5515,11 @@
       <c r="E169" s="3">
         <v>4428</v>
       </c>
-    </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F169" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="170" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A170" s="2" t="s">
         <v>345</v>
       </c>
@@ -5008,8 +5535,11 @@
       <c r="E170" s="3">
         <v>4428</v>
       </c>
-    </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F170" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="171" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A171" s="2" t="s">
         <v>347</v>
       </c>
@@ -5025,8 +5555,11 @@
       <c r="E171" s="3">
         <v>4428</v>
       </c>
-    </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F171" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="172" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A172" s="2" t="s">
         <v>349</v>
       </c>
@@ -5042,8 +5575,11 @@
       <c r="E172" s="3">
         <v>3330</v>
       </c>
-    </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F172" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="173" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A173" s="2" t="s">
         <v>351</v>
       </c>
@@ -5059,8 +5595,11 @@
       <c r="E173" s="3">
         <v>3330</v>
       </c>
-    </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F173" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="174" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A174" s="2" t="s">
         <v>353</v>
       </c>
@@ -5076,8 +5615,11 @@
       <c r="E174" s="3">
         <v>3330</v>
       </c>
-    </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F174" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="175" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A175" s="2" t="s">
         <v>355</v>
       </c>
@@ -5093,8 +5635,11 @@
       <c r="E175" s="3">
         <v>3330</v>
       </c>
-    </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F175" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="176" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A176" s="2" t="s">
         <v>357</v>
       </c>
@@ -5110,8 +5655,11 @@
       <c r="E176" s="3">
         <v>8238</v>
       </c>
-    </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F176" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="177" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A177" s="2" t="s">
         <v>359</v>
       </c>
@@ -5127,8 +5675,11 @@
       <c r="E177" s="3">
         <v>8238</v>
       </c>
-    </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F177" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="178" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A178" s="2" t="s">
         <v>361</v>
       </c>
@@ -5144,8 +5695,11 @@
       <c r="E178" s="3">
         <v>8238</v>
       </c>
-    </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F178" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="179" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A179" s="2" t="s">
         <v>363</v>
       </c>
@@ -5161,8 +5715,11 @@
       <c r="E179" s="3">
         <v>8238</v>
       </c>
-    </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F179" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="180" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A180" s="2" t="s">
         <v>365</v>
       </c>
@@ -5178,8 +5735,11 @@
       <c r="E180" s="3">
         <v>8238</v>
       </c>
-    </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F180" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="181" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A181" s="2" t="s">
         <v>367</v>
       </c>
@@ -5195,8 +5755,11 @@
       <c r="E181" s="3">
         <v>8238</v>
       </c>
-    </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F181" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="182" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A182" s="2" t="s">
         <v>369</v>
       </c>
@@ -5212,8 +5775,11 @@
       <c r="E182" s="3">
         <v>8238</v>
       </c>
-    </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F182" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="183" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A183" s="2" t="s">
         <v>371</v>
       </c>
@@ -5229,8 +5795,11 @@
       <c r="E183" s="3">
         <v>7550</v>
       </c>
-    </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F183" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="184" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A184" s="2" t="s">
         <v>373</v>
       </c>
@@ -5246,8 +5815,11 @@
       <c r="E184" s="3">
         <v>7550</v>
       </c>
-    </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F184" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="185" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A185" s="2" t="s">
         <v>375</v>
       </c>
@@ -5263,8 +5835,11 @@
       <c r="E185" s="3">
         <v>7550</v>
       </c>
-    </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F185" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="186" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A186" s="2" t="s">
         <v>377</v>
       </c>
@@ -5280,8 +5855,11 @@
       <c r="E186" s="3">
         <v>8280</v>
       </c>
-    </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F186" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="187" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A187" s="2" t="s">
         <v>379</v>
       </c>
@@ -5297,8 +5875,11 @@
       <c r="E187" s="3">
         <v>8280</v>
       </c>
-    </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F187" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="188" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A188" s="2" t="s">
         <v>381</v>
       </c>
@@ -5314,8 +5895,11 @@
       <c r="E188" s="3">
         <v>4750</v>
       </c>
-    </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F188" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="189" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A189" s="2" t="s">
         <v>383</v>
       </c>
@@ -5331,8 +5915,11 @@
       <c r="E189" s="3">
         <v>4866</v>
       </c>
-    </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F189" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="190" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A190" s="2" t="s">
         <v>385</v>
       </c>
@@ -5348,8 +5935,11 @@
       <c r="E190" s="3">
         <v>4866</v>
       </c>
-    </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F190" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="191" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A191" s="2" t="s">
         <v>387</v>
       </c>
@@ -5365,8 +5955,11 @@
       <c r="E191" s="3">
         <v>5940</v>
       </c>
-    </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F191" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="192" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A192" s="2" t="s">
         <v>389</v>
       </c>
@@ -5382,8 +5975,11 @@
       <c r="E192" s="3">
         <v>5940</v>
       </c>
-    </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F192" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="193" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A193" s="2" t="s">
         <v>391</v>
       </c>
@@ -5397,8 +5993,11 @@
         <v>394</v>
       </c>
       <c r="E193" s="3"/>
-    </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F193" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="194" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A194" s="2" t="s">
         <v>395</v>
       </c>
@@ -5412,8 +6011,11 @@
         <v>394</v>
       </c>
       <c r="E194" s="3"/>
-    </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F194" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="195" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A195" s="2" t="s">
         <v>397</v>
       </c>
@@ -5427,8 +6029,11 @@
         <v>394</v>
       </c>
       <c r="E195" s="3"/>
-    </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F195" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="196" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A196" s="2" t="s">
         <v>399</v>
       </c>
@@ -5444,8 +6049,11 @@
       <c r="E196" s="3">
         <v>17952</v>
       </c>
-    </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F196" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="197" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A197" s="2" t="s">
         <v>401</v>
       </c>
@@ -5461,8 +6069,11 @@
       <c r="E197" s="3">
         <v>17952</v>
       </c>
-    </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F197" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="198" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A198" s="2" t="s">
         <v>403</v>
       </c>
@@ -5478,8 +6089,11 @@
       <c r="E198" s="3">
         <v>17952</v>
       </c>
-    </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F198" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="199" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A199" s="2" t="s">
         <v>405</v>
       </c>
@@ -5495,8 +6109,11 @@
       <c r="E199" s="3">
         <v>17952</v>
       </c>
-    </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F199" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="200" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A200" s="2" t="s">
         <v>407</v>
       </c>
@@ -5512,8 +6129,11 @@
       <c r="E200" s="3">
         <v>17952</v>
       </c>
-    </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F200" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="201" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A201" s="2" t="s">
         <v>409</v>
       </c>
@@ -5529,8 +6149,11 @@
       <c r="E201" s="3">
         <v>17952</v>
       </c>
-    </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F201" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="202" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A202" s="2" t="s">
         <v>411</v>
       </c>
@@ -5546,8 +6169,11 @@
       <c r="E202" s="3">
         <v>17952</v>
       </c>
-    </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F202" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="203" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A203" s="2" t="s">
         <v>413</v>
       </c>
@@ -5563,8 +6189,11 @@
       <c r="E203" s="3">
         <v>13000</v>
       </c>
-    </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F203" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="204" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A204" s="2" t="s">
         <v>415</v>
       </c>
@@ -5580,8 +6209,11 @@
       <c r="E204" s="3">
         <v>13000</v>
       </c>
-    </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F204" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="205" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A205" s="2" t="s">
         <v>417</v>
       </c>
@@ -5597,8 +6229,11 @@
       <c r="E205" s="3">
         <v>13000</v>
       </c>
-    </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F205" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="206" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A206" s="2" t="s">
         <v>419</v>
       </c>
@@ -5614,8 +6249,11 @@
       <c r="E206" s="3">
         <v>18000</v>
       </c>
-    </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F206" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="207" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A207" s="2" t="s">
         <v>421</v>
       </c>
@@ -5631,8 +6269,11 @@
       <c r="E207" s="3">
         <v>18000</v>
       </c>
-    </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F207" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="208" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A208" s="2" t="s">
         <v>423</v>
       </c>
@@ -5648,8 +6289,11 @@
       <c r="E208" s="3">
         <v>18000</v>
       </c>
-    </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F208" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="209" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A209" s="2" t="s">
         <v>425</v>
       </c>
@@ -5665,8 +6309,11 @@
       <c r="E209" s="3">
         <v>3490</v>
       </c>
-    </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F209" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="210" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A210" s="2" t="s">
         <v>427</v>
       </c>
@@ -5682,8 +6329,11 @@
       <c r="E210" s="3">
         <v>3490</v>
       </c>
-    </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F210" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="211" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A211" s="2" t="s">
         <v>429</v>
       </c>
@@ -5699,8 +6349,11 @@
       <c r="E211" s="3">
         <v>3490</v>
       </c>
-    </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F211" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="212" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A212" s="2" t="s">
         <v>431</v>
       </c>
@@ -5716,8 +6369,11 @@
       <c r="E212" s="3">
         <v>3490</v>
       </c>
-    </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F212" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="213" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A213" s="2" t="s">
         <v>433</v>
       </c>
@@ -5733,8 +6389,11 @@
       <c r="E213" s="3">
         <v>3490</v>
       </c>
-    </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F213" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="214" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A214" s="2" t="s">
         <v>435</v>
       </c>
@@ -5750,8 +6409,11 @@
       <c r="E214" s="3">
         <v>3490</v>
       </c>
-    </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F214" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="215" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A215" s="2" t="s">
         <v>437</v>
       </c>
@@ -5767,8 +6429,11 @@
       <c r="E215" s="3">
         <v>3490</v>
       </c>
-    </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F215" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="216" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A216" s="2" t="s">
         <v>439</v>
       </c>
@@ -5784,8 +6449,11 @@
       <c r="E216" s="3">
         <v>3590</v>
       </c>
-    </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F216" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="217" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A217" s="2" t="s">
         <v>441</v>
       </c>
@@ -5801,8 +6469,11 @@
       <c r="E217" s="3">
         <v>3590</v>
       </c>
-    </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F217" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="218" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A218" s="2" t="s">
         <v>443</v>
       </c>
@@ -5818,8 +6489,11 @@
       <c r="E218" s="3">
         <v>3590</v>
       </c>
-    </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F218" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="219" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A219" s="2" t="s">
         <v>445</v>
       </c>
@@ -5835,8 +6509,11 @@
       <c r="E219" s="3">
         <v>3590</v>
       </c>
-    </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F219" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="220" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A220" s="2" t="s">
         <v>447</v>
       </c>
@@ -5852,8 +6529,11 @@
       <c r="E220" s="3">
         <v>3590</v>
       </c>
-    </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F220" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="221" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A221" s="2" t="s">
         <v>449</v>
       </c>
@@ -5869,8 +6549,11 @@
       <c r="E221" s="3">
         <v>3590</v>
       </c>
-    </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F221" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="222" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A222" s="2" t="s">
         <v>451</v>
       </c>
@@ -5886,8 +6569,11 @@
       <c r="E222" s="3">
         <v>3590</v>
       </c>
-    </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F222" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="223" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A223" s="2" t="s">
         <v>391</v>
       </c>
@@ -5901,8 +6587,11 @@
         <v>394</v>
       </c>
       <c r="E223" s="3"/>
-    </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F223" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="224" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A224" s="2" t="s">
         <v>395</v>
       </c>
@@ -5916,8 +6605,11 @@
         <v>394</v>
       </c>
       <c r="E224" s="3"/>
-    </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F224" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="225" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A225" s="2" t="s">
         <v>397</v>
       </c>
@@ -5931,8 +6623,11 @@
         <v>394</v>
       </c>
       <c r="E225" s="3"/>
-    </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F225" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="226" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A226" s="2" t="s">
         <v>456</v>
       </c>
@@ -5948,8 +6643,11 @@
       <c r="E226" s="3">
         <v>19680</v>
       </c>
-    </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F226" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="227" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A227" s="2" t="s">
         <v>458</v>
       </c>
@@ -5965,8 +6663,11 @@
       <c r="E227" s="3">
         <v>19680</v>
       </c>
-    </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F227" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="228" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A228" s="2" t="s">
         <v>460</v>
       </c>
@@ -5982,8 +6683,11 @@
       <c r="E228" s="3">
         <v>19680</v>
       </c>
-    </row>
-    <row r="229" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F228" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="229" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A229" s="2" t="s">
         <v>462</v>
       </c>
@@ -5999,8 +6703,11 @@
       <c r="E229" s="3">
         <v>19680</v>
       </c>
-    </row>
-    <row r="230" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F229" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="230" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A230" s="2" t="s">
         <v>464</v>
       </c>
@@ -6016,8 +6723,11 @@
       <c r="E230" s="3">
         <v>19680</v>
       </c>
-    </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F230" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="231" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A231" s="2" t="s">
         <v>466</v>
       </c>
@@ -6033,8 +6743,11 @@
       <c r="E231" s="3">
         <v>19680</v>
       </c>
-    </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F231" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="232" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A232" s="2" t="s">
         <v>468</v>
       </c>
@@ -6050,8 +6763,11 @@
       <c r="E232" s="3">
         <v>19680</v>
       </c>
-    </row>
-    <row r="233" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F232" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="233" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A233" s="2" t="s">
         <v>470</v>
       </c>
@@ -6067,8 +6783,11 @@
       <c r="E233" s="3">
         <v>19680</v>
       </c>
-    </row>
-    <row r="234" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F233" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="234" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A234" s="2" t="s">
         <v>472</v>
       </c>
@@ -6084,8 +6803,11 @@
       <c r="E234" s="3">
         <v>9000</v>
       </c>
-    </row>
-    <row r="235" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F234" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="235" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A235" s="2" t="s">
         <v>475</v>
       </c>
@@ -6101,8 +6823,11 @@
       <c r="E235" s="3">
         <v>9000</v>
       </c>
-    </row>
-    <row r="236" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F235" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="236" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A236" s="2" t="s">
         <v>477</v>
       </c>
@@ -6118,8 +6843,11 @@
       <c r="E236" s="3">
         <v>9000</v>
       </c>
-    </row>
-    <row r="237" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F236" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="237" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A237" s="2" t="s">
         <v>479</v>
       </c>
@@ -6135,8 +6863,11 @@
       <c r="E237" s="3">
         <v>9000</v>
       </c>
-    </row>
-    <row r="238" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F237" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="238" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A238" s="2" t="s">
         <v>481</v>
       </c>
@@ -6152,8 +6883,11 @@
       <c r="E238" s="3">
         <v>9300</v>
       </c>
-    </row>
-    <row r="239" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F238" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="239" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A239" s="2" t="s">
         <v>483</v>
       </c>
@@ -6169,8 +6903,11 @@
       <c r="E239" s="3">
         <v>9300</v>
       </c>
-    </row>
-    <row r="240" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F239" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="240" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A240" s="2" t="s">
         <v>485</v>
       </c>
@@ -6186,8 +6923,11 @@
       <c r="E240" s="3">
         <v>9300</v>
       </c>
-    </row>
-    <row r="241" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F240" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="241" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A241" s="2" t="s">
         <v>487</v>
       </c>
@@ -6203,8 +6943,11 @@
       <c r="E241" s="3">
         <v>5760</v>
       </c>
-    </row>
-    <row r="242" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F241" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="242" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A242" s="2" t="s">
         <v>489</v>
       </c>
@@ -6220,8 +6963,11 @@
       <c r="E242" s="3">
         <v>5760</v>
       </c>
-    </row>
-    <row r="243" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F242" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="243" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A243" s="2" t="s">
         <v>491</v>
       </c>
@@ -6237,8 +6983,11 @@
       <c r="E243" s="3">
         <v>5760</v>
       </c>
-    </row>
-    <row r="244" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F243" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="244" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A244" s="2" t="s">
         <v>493</v>
       </c>
@@ -6254,8 +7003,11 @@
       <c r="E244" s="3">
         <v>5760</v>
       </c>
-    </row>
-    <row r="245" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F244" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="245" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A245" s="2" t="s">
         <v>495</v>
       </c>
@@ -6271,8 +7023,11 @@
       <c r="E245" s="3">
         <v>5760</v>
       </c>
-    </row>
-    <row r="246" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F245" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="246" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A246" s="2" t="s">
         <v>497</v>
       </c>
@@ -6288,8 +7043,11 @@
       <c r="E246" s="3">
         <v>5760</v>
       </c>
-    </row>
-    <row r="247" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F246" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="247" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A247" s="2" t="s">
         <v>499</v>
       </c>
@@ -6305,8 +7063,11 @@
       <c r="E247" s="3">
         <v>19000</v>
       </c>
-    </row>
-    <row r="248" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F247" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="248" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A248" s="2" t="s">
         <v>503</v>
       </c>
@@ -6322,8 +7083,11 @@
       <c r="E248" s="3">
         <v>19000</v>
       </c>
-    </row>
-    <row r="249" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F248" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="249" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A249" s="2" t="s">
         <v>505</v>
       </c>
@@ -6339,8 +7103,11 @@
       <c r="E249" s="3">
         <v>19000</v>
       </c>
-    </row>
-    <row r="250" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F249" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="250" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A250" s="2" t="s">
         <v>507</v>
       </c>
@@ -6356,8 +7123,11 @@
       <c r="E250" s="3">
         <v>19000</v>
       </c>
-    </row>
-    <row r="251" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F250" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="251" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A251" s="2" t="s">
         <v>509</v>
       </c>
@@ -6373,8 +7143,11 @@
       <c r="E251" s="3">
         <v>4500</v>
       </c>
-    </row>
-    <row r="252" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F251" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="252" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A252" s="2" t="s">
         <v>511</v>
       </c>
@@ -6390,8 +7163,11 @@
       <c r="E252" s="3">
         <v>4500</v>
       </c>
-    </row>
-    <row r="253" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F252" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="253" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A253" s="2" t="s">
         <v>513</v>
       </c>
@@ -6407,8 +7183,11 @@
       <c r="E253" s="3">
         <v>4500</v>
       </c>
-    </row>
-    <row r="254" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F253" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="254" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A254" s="2" t="s">
         <v>515</v>
       </c>
@@ -6424,8 +7203,11 @@
       <c r="E254" s="3">
         <v>4250</v>
       </c>
-    </row>
-    <row r="255" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F254" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="255" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A255" s="2" t="s">
         <v>517</v>
       </c>
@@ -6441,8 +7223,11 @@
       <c r="E255" s="3">
         <v>4250</v>
       </c>
-    </row>
-    <row r="256" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F255" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="256" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A256" s="2" t="s">
         <v>519</v>
       </c>
@@ -6458,8 +7243,11 @@
       <c r="E256" s="3">
         <v>4250</v>
       </c>
-    </row>
-    <row r="257" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F256" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="257" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A257" s="2" t="s">
         <v>521</v>
       </c>
@@ -6475,8 +7263,11 @@
       <c r="E257" s="3">
         <v>4250</v>
       </c>
-    </row>
-    <row r="258" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F257" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="258" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A258" s="2" t="s">
         <v>523</v>
       </c>
@@ -6492,8 +7283,11 @@
       <c r="E258" s="3">
         <v>15650</v>
       </c>
-    </row>
-    <row r="259" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F258" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="259" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A259" s="2" t="s">
         <v>525</v>
       </c>
@@ -6509,8 +7303,11 @@
       <c r="E259" s="3">
         <v>15650</v>
       </c>
-    </row>
-    <row r="260" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F259" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="260" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A260" s="2" t="s">
         <v>527</v>
       </c>
@@ -6526,8 +7323,11 @@
       <c r="E260" s="3">
         <v>15650</v>
       </c>
-    </row>
-    <row r="261" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F260" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="261" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A261" s="2" t="s">
         <v>529</v>
       </c>
@@ -6543,8 +7343,11 @@
       <c r="E261" s="3">
         <v>15650</v>
       </c>
-    </row>
-    <row r="262" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F261" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="262" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A262" s="2" t="s">
         <v>531</v>
       </c>
@@ -6560,8 +7363,11 @@
       <c r="E262" s="3">
         <v>15650</v>
       </c>
-    </row>
-    <row r="263" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F262" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="263" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A263" s="2" t="s">
         <v>533</v>
       </c>
@@ -6577,8 +7383,11 @@
       <c r="E263" s="3">
         <v>15650</v>
       </c>
-    </row>
-    <row r="264" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F263" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="264" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A264" s="2" t="s">
         <v>535</v>
       </c>
@@ -6594,8 +7403,11 @@
       <c r="E264" s="3">
         <v>5800</v>
       </c>
-    </row>
-    <row r="265" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F264" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="265" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A265" s="2" t="s">
         <v>537</v>
       </c>
@@ -6611,8 +7423,11 @@
       <c r="E265" s="3">
         <v>5800</v>
       </c>
-    </row>
-    <row r="266" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F265" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="266" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A266" s="2" t="s">
         <v>539</v>
       </c>
@@ -6628,8 +7443,11 @@
       <c r="E266" s="3">
         <v>5800</v>
       </c>
-    </row>
-    <row r="267" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F266" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="267" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A267" s="2" t="s">
         <v>541</v>
       </c>
@@ -6645,8 +7463,11 @@
       <c r="E267" s="3">
         <v>5800</v>
       </c>
-    </row>
-    <row r="268" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F267" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="268" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A268" s="2" t="s">
         <v>543</v>
       </c>
@@ -6662,8 +7483,11 @@
       <c r="E268" s="3">
         <v>3590</v>
       </c>
-    </row>
-    <row r="269" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F268" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="269" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A269" s="2" t="s">
         <v>545</v>
       </c>
@@ -6679,8 +7503,11 @@
       <c r="E269" s="3">
         <v>3590</v>
       </c>
-    </row>
-    <row r="270" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F269" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="270" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A270" s="2" t="s">
         <v>547</v>
       </c>
@@ -6696,8 +7523,11 @@
       <c r="E270" s="3">
         <v>17880</v>
       </c>
-    </row>
-    <row r="271" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F270" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="271" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A271" s="2" t="s">
         <v>549</v>
       </c>
@@ -6713,8 +7543,11 @@
       <c r="E271" s="3">
         <v>7900</v>
       </c>
-    </row>
-    <row r="272" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F271" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="272" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A272" s="2" t="s">
         <v>551</v>
       </c>
@@ -6730,8 +7563,11 @@
       <c r="E272" s="3">
         <v>7900</v>
       </c>
-    </row>
-    <row r="273" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F272" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="273" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A273" s="2" t="s">
         <v>553</v>
       </c>
@@ -6747,8 +7583,11 @@
       <c r="E273" s="3">
         <v>7900</v>
       </c>
-    </row>
-    <row r="274" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F273" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="274" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A274" s="2" t="s">
         <v>555</v>
       </c>
@@ -6764,8 +7603,11 @@
       <c r="E274" s="3">
         <v>15600</v>
       </c>
-    </row>
-    <row r="275" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F274" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="275" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A275" s="2" t="s">
         <v>557</v>
       </c>
@@ -6781,8 +7623,11 @@
       <c r="E275" s="3">
         <v>15600</v>
       </c>
-    </row>
-    <row r="276" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F275" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="276" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A276" s="2" t="s">
         <v>559</v>
       </c>
@@ -6798,8 +7643,11 @@
       <c r="E276" s="3">
         <v>6950</v>
       </c>
-    </row>
-    <row r="277" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F276" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="277" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A277" s="2" t="s">
         <v>563</v>
       </c>
@@ -6815,8 +7663,11 @@
       <c r="E277" s="3">
         <v>36000</v>
       </c>
-    </row>
-    <row r="278" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F277" s="5">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="278" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A278" s="2" t="s">
         <v>566</v>
       </c>
@@ -6831,6 +7682,9 @@
       </c>
       <c r="E278" s="3">
         <v>32000</v>
+      </c>
+      <c r="F278" s="5">
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>